<commit_message>
add power of attorney
</commit_message>
<xml_diff>
--- a/docs/CodeSystem-AuthorizedCodes.xlsx
+++ b/docs/CodeSystem-AuthorizedCodes.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="46">
   <si>
     <t>Property</t>
   </si>
@@ -27,6 +27,12 @@
     <t>http://johnmoehrke.github.io/RelatedPersonConsent/CodeSystem/AuthorizedCodes</t>
   </si>
   <si>
+    <t>Identifier</t>
+  </si>
+  <si>
+    <t>OID:1.3.6.1.4.1.66281.5.16.1</t>
+  </si>
+  <si>
     <t>Version</t>
   </si>
   <si>
@@ -54,10 +60,13 @@
     <t>Experimental</t>
   </si>
   <si>
+    <t>false</t>
+  </si>
+  <si>
     <t>Date</t>
   </si>
   <si>
-    <t>2022-06-17T07:29:17-05:00</t>
+    <t>2026-08-18T10:19:00-05:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -69,13 +78,16 @@
     <t>Contact</t>
   </si>
   <si>
-    <t>No display for ContactDetail</t>
+    <t>John Moehrke (himself) (http://healthcaresecprivacy.blogspot.com, JohnMoehrke@gmail.com)</t>
+  </si>
+  <si>
+    <t>John Moehrke (himself) (JohnMoehrke@gmail.com)</t>
   </si>
   <si>
     <t>Jurisdiction</t>
   </si>
   <si>
-    <t>World</t>
+    <t>Global (Whole world)</t>
   </si>
   <si>
     <t>Description</t>
@@ -260,10 +272,10 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyBorder="true" applyFill="true" applyFont="true">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyBorder="true" applyFill="true" applyAlignment="true" applyFont="true">
       <alignment vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="true">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="true" applyAlignment="true">
       <alignment vertical="top" wrapText="true"/>
     </xf>
   </cellXfs>
@@ -272,7 +284,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="15.703125" customWidth="true"/>
@@ -331,120 +343,130 @@
       <c r="A7" t="s" s="2">
         <v>12</v>
       </c>
-      <c r="B7" s="2"/>
+      <c r="B7" t="s" s="2">
+        <v>13</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="2">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B8" t="s" s="2">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="2">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B9" t="s" s="2">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="2">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B10" t="s" s="2">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="2">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B11" t="s" s="2">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="2">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="2">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
-        <v>23</v>
-      </c>
-      <c r="B14" s="2"/>
+        <v>25</v>
+      </c>
+      <c r="B14" t="s" s="2">
+        <v>26</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="2">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B15" s="2"/>
     </row>
     <row r="16">
       <c r="A16" t="s" s="2">
-        <v>25</v>
-      </c>
-      <c r="B16" t="s" s="2">
-        <v>26</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="B16" s="2"/>
     </row>
     <row r="17">
       <c r="A17" t="s" s="2">
-        <v>27</v>
-      </c>
-      <c r="B17" s="2"/>
+        <v>29</v>
+      </c>
+      <c r="B17" t="s" s="2">
+        <v>30</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="2">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B18" s="2"/>
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B19" s="2"/>
     </row>
     <row r="20">
       <c r="A20" t="s" s="2">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B20" s="2"/>
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
-        <v>31</v>
-      </c>
-      <c r="B21" t="s" s="2">
-        <v>32</v>
-      </c>
+        <v>34</v>
+      </c>
+      <c r="B21" s="2"/>
     </row>
     <row r="22">
       <c r="A22" t="s" s="2">
-        <v>33</v>
-      </c>
-      <c r="B22" s="2"/>
+        <v>35</v>
+      </c>
+      <c r="B22" t="s" s="2">
+        <v>36</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="2">
-        <v>34</v>
-      </c>
-      <c r="B23" t="s" s="2">
-        <v>35</v>
+        <v>37</v>
+      </c>
+      <c r="B23" s="2"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="s" s="2">
+        <v>38</v>
+      </c>
+      <c r="B24" t="s" s="2">
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -459,27 +481,27 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="1">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B1" t="s" s="1">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C1" t="s" s="1">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D1" t="s" s="1">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="2">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="B2" t="s" s="2">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="C2" t="s" s="2">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="D2" s="2"/>
     </row>

</xml_diff>